<commit_message>
Actualización de estatus de pólizas (activos e inactivos)
</commit_message>
<xml_diff>
--- a/mdrt/MDRT.xlsx
+++ b/mdrt/MDRT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/mdrt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F831C410-6B00-8C4F-9081-628C0ED4BC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A19AB92-40C5-C140-B632-93C170C618C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{263D14F0-BAEF-1E4F-83AF-E2F80B31AC70}"/>
   </bookViews>
@@ -782,76 +782,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="49">
-    <dxf>
-      <border>
-        <left style="hair">
-          <color rgb="FF002060"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF002060"/>
-        </right>
-        <top style="hair">
-          <color rgb="FF002060"/>
-        </top>
-        <bottom style="hair">
-          <color rgb="FF002060"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color rgb="FF002060"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF002060"/>
-        </right>
-        <top style="hair">
-          <color rgb="FF002060"/>
-        </top>
-        <bottom style="hair">
-          <color rgb="FF002060"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="45">
     <dxf>
       <fill>
         <patternFill>
@@ -1973,49 +1904,49 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BCF95067-B771-3C4D-AD63-C29CB67B4C88}" name="Tabla1" displayName="Tabla1" ref="A4:AN53" totalsRowShown="0" dataDxfId="48" dataCellStyle="Millares">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BCF95067-B771-3C4D-AD63-C29CB67B4C88}" name="Tabla1" displayName="Tabla1" ref="A4:AN53" totalsRowShown="0" dataDxfId="44" dataCellStyle="Millares">
   <autoFilter ref="A4:AN53" xr:uid="{BCF95067-B771-3C4D-AD63-C29CB67B4C88}"/>
   <tableColumns count="40">
-    <tableColumn id="1" xr3:uid="{1B45D68F-9E92-9A48-B147-43382D17EADB}" name="Dir / Zona" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{8141432D-DFE6-034B-8474-F9783519965C}" name="Oficina" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{3026117E-099F-6549-A16F-3CA4F85DA282}" name="Mat" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{80621F5B-C573-8944-AF37-DC364F1BE0A9}" name="Suc" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{9D7D11D1-2D98-5646-92D8-F8703E85240A}" name="Promotor / Partner" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{870F3B42-A14B-1947-827D-9A6082152D25}" name="Asesor" dataDxfId="42"/>
-    <tableColumn id="7" xr3:uid="{CA38BEAA-FBC9-474E-8C66-960105DEBCF2}" name="Nombre del Asesor" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{8B8898BF-4E49-0543-9598-18FF2D3F6340}" name="Conexión" dataDxfId="40"/>
-    <tableColumn id="9" xr3:uid="{49ED1251-337D-EC49-A858-207AB60B673C}" name="Grupo" dataDxfId="39" dataCellStyle="Millares"/>
-    <tableColumn id="10" xr3:uid="{26692A66-EA2C-DD40-AAC8-07A5FE32BC7D}" name="Vida Individual" dataDxfId="38" dataCellStyle="Millares"/>
-    <tableColumn id="11" xr3:uid="{45DC445E-D43B-394B-91CD-B3001CC307CC}" name="Vida G&amp;C" dataDxfId="37" dataCellStyle="Millares"/>
-    <tableColumn id="12" xr3:uid="{953B1F2A-AB88-8A40-B82F-B5DBE8FAEA70}" name="Segudescuento" dataDxfId="36" dataCellStyle="Millares"/>
-    <tableColumn id="13" xr3:uid="{27E03CF4-3925-2045-BF66-C5BB1ECC7061}" name="Aportaciones Adicionales (AVEs)" dataDxfId="35" dataCellStyle="Millares"/>
-    <tableColumn id="14" xr3:uid="{7375183C-90AB-0B47-A516-65079E7802F1}" name="Cancelacion de Pólizas" dataDxfId="34" dataCellStyle="Millares"/>
-    <tableColumn id="15" xr3:uid="{B0F3DBFB-9B00-894E-8929-BF5CA63336C6}" name="Total de Productos Ilimitados" dataDxfId="33" dataCellStyle="Millares"/>
-    <tableColumn id="16" xr3:uid="{3C9D5C71-B64C-434C-8D65-968245DAE09C}" name="%Vida vs Meta" dataDxfId="32" dataCellStyle="Porcentaje"/>
-    <tableColumn id="17" xr3:uid="{088A86A3-8B28-DE4E-A384-CA0EA913DA34}" name="GMM Individual" dataDxfId="31" dataCellStyle="Millares"/>
-    <tableColumn id="18" xr3:uid="{A8791E9D-69D9-C844-AE4C-8AEEFA976B8B}" name="GMM G&amp;C" dataDxfId="30" dataCellStyle="Millares"/>
-    <tableColumn id="19" xr3:uid="{0FFCB5A1-F8D9-2344-9DC7-667454959C98}" name="Cancelacion de Pólizas2" dataDxfId="29" dataCellStyle="Millares"/>
-    <tableColumn id="20" xr3:uid="{FDCA43A0-92B9-954B-B283-ABAD7C194405}" name="Total Productos Limitados" dataDxfId="28" dataCellStyle="Millares"/>
-    <tableColumn id="21" xr3:uid="{7C93BB8B-9213-EA49-A648-EF5192999BF7}" name="Tope personales" dataDxfId="27" dataCellStyle="Millares"/>
-    <tableColumn id="22" xr3:uid="{70D3FAB6-79FB-994B-AB69-F0BBB15C6AFD}" name="Total Prima" dataDxfId="26" dataCellStyle="Millares"/>
-    <tableColumn id="23" xr3:uid="{0E0D17EB-06B5-AF45-9773-7D3921FC5B9C}" name="Vida Individual3" dataDxfId="25" dataCellStyle="Millares"/>
-    <tableColumn id="24" xr3:uid="{2A25EC7F-F387-9948-8D9A-38BFD2316AB4}" name="Vida G&amp;C4" dataDxfId="24" dataCellStyle="Millares"/>
-    <tableColumn id="25" xr3:uid="{F7E8005C-762C-7146-A541-3589C41B3DA2}" name="Segudescuento5" dataDxfId="23" dataCellStyle="Millares"/>
-    <tableColumn id="26" xr3:uid="{278BB65E-357A-1D4C-B1D0-5880BBD354CD}" name="Aportaciones Adicionales (AVEs)6" dataDxfId="22" dataCellStyle="Millares"/>
-    <tableColumn id="27" xr3:uid="{0490A388-0C84-C043-A7E8-E5DC8A03AF3F}" name="Cancelacion de Pólizas7" dataDxfId="21" dataCellStyle="Millares"/>
-    <tableColumn id="28" xr3:uid="{C06E1BE2-8968-A045-B8AB-E420B9B469A1}" name="Total de Productos Ilimitados8" dataDxfId="20" dataCellStyle="Millares"/>
-    <tableColumn id="29" xr3:uid="{BEBE08BA-F641-3141-BCA9-713FD1C7CEC2}" name="%Vida vs Meta9" dataDxfId="19" dataCellStyle="Porcentaje"/>
-    <tableColumn id="30" xr3:uid="{E7FB912B-27FD-1345-845F-E51E648031F5}" name="GMM Individual10" dataDxfId="18" dataCellStyle="Millares"/>
-    <tableColumn id="31" xr3:uid="{D5FF299C-A405-CE44-B4CD-CED400EFE81F}" name="GMM G&amp;C11" dataDxfId="17" dataCellStyle="Millares"/>
-    <tableColumn id="32" xr3:uid="{D7EFF89B-8E34-EA46-B72C-61EE3166E416}" name="Cancelacion de Pólizas12" dataDxfId="16" dataCellStyle="Millares"/>
-    <tableColumn id="33" xr3:uid="{81E1798B-3D20-E748-BDAB-7A2A6F5BF33B}" name="Total Productos Limitados13" dataDxfId="15" dataCellStyle="Millares"/>
-    <tableColumn id="34" xr3:uid="{7A820362-E31F-4D41-B400-9AD11AE00577}" name="Tope personales14" dataDxfId="14" dataCellStyle="Millares"/>
-    <tableColumn id="35" xr3:uid="{09E5F95B-08D0-B946-B14E-3F06BC9C57F0}" name="Total Comisión" dataDxfId="13" dataCellStyle="Millares"/>
-    <tableColumn id="36" xr3:uid="{523C81DC-6FA9-A24D-AF9B-9D74B552A8BA}" name="Columna15" dataDxfId="12" dataCellStyle="Millares"/>
-    <tableColumn id="37" xr3:uid="{ACF68D6F-CC4F-F94A-A3AE-C7407A1AC3DE}" name="Camino Prima" dataDxfId="11" dataCellStyle="Millares"/>
-    <tableColumn id="38" xr3:uid="{39FE9301-7AE9-0A42-B79D-CA4998AB76AE}" name="OBSERVACIÓN" dataDxfId="10" dataCellStyle="Millares"/>
-    <tableColumn id="39" xr3:uid="{99E25200-803C-E54D-88BD-27CB86CAED40}" name="Camino  Comisión" dataDxfId="9" dataCellStyle="Millares"/>
-    <tableColumn id="40" xr3:uid="{45B29C50-720D-8F4E-9803-310BA4AC814E}" name="NIVEL_x000a_" dataDxfId="8" dataCellStyle="Millares"/>
+    <tableColumn id="1" xr3:uid="{1B45D68F-9E92-9A48-B147-43382D17EADB}" name="Dir / Zona" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{8141432D-DFE6-034B-8474-F9783519965C}" name="Oficina" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{3026117E-099F-6549-A16F-3CA4F85DA282}" name="Mat" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{80621F5B-C573-8944-AF37-DC364F1BE0A9}" name="Suc" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{9D7D11D1-2D98-5646-92D8-F8703E85240A}" name="Promotor / Partner" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{870F3B42-A14B-1947-827D-9A6082152D25}" name="Asesor" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{CA38BEAA-FBC9-474E-8C66-960105DEBCF2}" name="Nombre del Asesor" dataDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{8B8898BF-4E49-0543-9598-18FF2D3F6340}" name="Conexión" dataDxfId="36"/>
+    <tableColumn id="9" xr3:uid="{49ED1251-337D-EC49-A858-207AB60B673C}" name="Grupo" dataDxfId="35" dataCellStyle="Millares"/>
+    <tableColumn id="10" xr3:uid="{26692A66-EA2C-DD40-AAC8-07A5FE32BC7D}" name="Vida Individual" dataDxfId="34" dataCellStyle="Millares"/>
+    <tableColumn id="11" xr3:uid="{45DC445E-D43B-394B-91CD-B3001CC307CC}" name="Vida G&amp;C" dataDxfId="33" dataCellStyle="Millares"/>
+    <tableColumn id="12" xr3:uid="{953B1F2A-AB88-8A40-B82F-B5DBE8FAEA70}" name="Segudescuento" dataDxfId="32" dataCellStyle="Millares"/>
+    <tableColumn id="13" xr3:uid="{27E03CF4-3925-2045-BF66-C5BB1ECC7061}" name="Aportaciones Adicionales (AVEs)" dataDxfId="31" dataCellStyle="Millares"/>
+    <tableColumn id="14" xr3:uid="{7375183C-90AB-0B47-A516-65079E7802F1}" name="Cancelacion de Pólizas" dataDxfId="30" dataCellStyle="Millares"/>
+    <tableColumn id="15" xr3:uid="{B0F3DBFB-9B00-894E-8929-BF5CA63336C6}" name="Total de Productos Ilimitados" dataDxfId="29" dataCellStyle="Millares"/>
+    <tableColumn id="16" xr3:uid="{3C9D5C71-B64C-434C-8D65-968245DAE09C}" name="%Vida vs Meta" dataDxfId="28" dataCellStyle="Porcentaje"/>
+    <tableColumn id="17" xr3:uid="{088A86A3-8B28-DE4E-A384-CA0EA913DA34}" name="GMM Individual" dataDxfId="27" dataCellStyle="Millares"/>
+    <tableColumn id="18" xr3:uid="{A8791E9D-69D9-C844-AE4C-8AEEFA976B8B}" name="GMM G&amp;C" dataDxfId="26" dataCellStyle="Millares"/>
+    <tableColumn id="19" xr3:uid="{0FFCB5A1-F8D9-2344-9DC7-667454959C98}" name="Cancelacion de Pólizas2" dataDxfId="25" dataCellStyle="Millares"/>
+    <tableColumn id="20" xr3:uid="{FDCA43A0-92B9-954B-B283-ABAD7C194405}" name="Total Productos Limitados" dataDxfId="24" dataCellStyle="Millares"/>
+    <tableColumn id="21" xr3:uid="{7C93BB8B-9213-EA49-A648-EF5192999BF7}" name="Tope personales" dataDxfId="23" dataCellStyle="Millares"/>
+    <tableColumn id="22" xr3:uid="{70D3FAB6-79FB-994B-AB69-F0BBB15C6AFD}" name="Total Prima" dataDxfId="22" dataCellStyle="Millares"/>
+    <tableColumn id="23" xr3:uid="{0E0D17EB-06B5-AF45-9773-7D3921FC5B9C}" name="Vida Individual3" dataDxfId="21" dataCellStyle="Millares"/>
+    <tableColumn id="24" xr3:uid="{2A25EC7F-F387-9948-8D9A-38BFD2316AB4}" name="Vida G&amp;C4" dataDxfId="20" dataCellStyle="Millares"/>
+    <tableColumn id="25" xr3:uid="{F7E8005C-762C-7146-A541-3589C41B3DA2}" name="Segudescuento5" dataDxfId="19" dataCellStyle="Millares"/>
+    <tableColumn id="26" xr3:uid="{278BB65E-357A-1D4C-B1D0-5880BBD354CD}" name="Aportaciones Adicionales (AVEs)6" dataDxfId="18" dataCellStyle="Millares"/>
+    <tableColumn id="27" xr3:uid="{0490A388-0C84-C043-A7E8-E5DC8A03AF3F}" name="Cancelacion de Pólizas7" dataDxfId="17" dataCellStyle="Millares"/>
+    <tableColumn id="28" xr3:uid="{C06E1BE2-8968-A045-B8AB-E420B9B469A1}" name="Total de Productos Ilimitados8" dataDxfId="16" dataCellStyle="Millares"/>
+    <tableColumn id="29" xr3:uid="{BEBE08BA-F641-3141-BCA9-713FD1C7CEC2}" name="%Vida vs Meta9" dataDxfId="15" dataCellStyle="Porcentaje"/>
+    <tableColumn id="30" xr3:uid="{E7FB912B-27FD-1345-845F-E51E648031F5}" name="GMM Individual10" dataDxfId="14" dataCellStyle="Millares"/>
+    <tableColumn id="31" xr3:uid="{D5FF299C-A405-CE44-B4CD-CED400EFE81F}" name="GMM G&amp;C11" dataDxfId="13" dataCellStyle="Millares"/>
+    <tableColumn id="32" xr3:uid="{D7EFF89B-8E34-EA46-B72C-61EE3166E416}" name="Cancelacion de Pólizas12" dataDxfId="12" dataCellStyle="Millares"/>
+    <tableColumn id="33" xr3:uid="{81E1798B-3D20-E748-BDAB-7A2A6F5BF33B}" name="Total Productos Limitados13" dataDxfId="11" dataCellStyle="Millares"/>
+    <tableColumn id="34" xr3:uid="{7A820362-E31F-4D41-B400-9AD11AE00577}" name="Tope personales14" dataDxfId="10" dataCellStyle="Millares"/>
+    <tableColumn id="35" xr3:uid="{09E5F95B-08D0-B946-B14E-3F06BC9C57F0}" name="Total Comisión" dataDxfId="9" dataCellStyle="Millares"/>
+    <tableColumn id="36" xr3:uid="{523C81DC-6FA9-A24D-AF9B-9D74B552A8BA}" name="Columna15" dataDxfId="8" dataCellStyle="Millares"/>
+    <tableColumn id="37" xr3:uid="{ACF68D6F-CC4F-F94A-A3AE-C7407A1AC3DE}" name="Camino Prima" dataDxfId="7" dataCellStyle="Millares"/>
+    <tableColumn id="38" xr3:uid="{39FE9301-7AE9-0A42-B79D-CA4998AB76AE}" name="OBSERVACIÓN" dataDxfId="6" dataCellStyle="Millares"/>
+    <tableColumn id="39" xr3:uid="{99E25200-803C-E54D-88BD-27CB86CAED40}" name="Camino  Comisión" dataDxfId="5" dataCellStyle="Millares"/>
+    <tableColumn id="40" xr3:uid="{45B29C50-720D-8F4E-9803-310BA4AC814E}" name="NIVEL_x000a_" dataDxfId="4" dataCellStyle="Millares"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7954,44 +7885,24 @@
       <c r="AN53" s="35"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A53:AI53 AM53:AN53 AK53">
-    <cfRule type="expression" dxfId="7" priority="9" stopIfTrue="1">
-      <formula>$B53&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK53:AN53">
-    <cfRule type="expression" dxfId="6" priority="5" stopIfTrue="1">
-      <formula>$B53&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL53">
-    <cfRule type="expression" dxfId="5" priority="7" stopIfTrue="1">
-      <formula>$B53&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AN53 V53 AI53">
-    <cfRule type="expression" dxfId="4" priority="8" stopIfTrue="1">
-      <formula>$B53&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6:AI52 AK6:AK52 AM6:AN52">
+  <conditionalFormatting sqref="A6:AI53 AM6:AN53 AK6:AK53">
     <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:V52 AI6:AI52 AN6:AN52">
-    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
-      <formula>$B6&lt;&gt;""</formula>
+  <conditionalFormatting sqref="AK42:AN53">
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
+      <formula>$B42&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL6:AL52">
+  <conditionalFormatting sqref="AL6:AL53">
     <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK42:AN52">
-    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>$B42&lt;&gt;""</formula>
+  <conditionalFormatting sqref="AN6:AN53 V6:V53 AI6:AI53">
+    <cfRule type="expression" dxfId="0" priority="3" stopIfTrue="1">
+      <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-20 09:22)
</commit_message>
<xml_diff>
--- a/mdrt/MDRT.xlsx
+++ b/mdrt/MDRT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/mdrt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEFE5E8F-1F47-2343-973D-98C2FD681F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D04F39-F1A7-574A-A1F4-FB1A39450675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{263D14F0-BAEF-1E4F-83AF-E2F80B31AC70}"/>
   </bookViews>
@@ -776,92 +776,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="50">
-    <dxf>
-      <border>
-        <left style="hair">
-          <color rgb="FF002060"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF002060"/>
-        </right>
-        <top style="hair">
-          <color rgb="FF002060"/>
-        </top>
-        <bottom style="hair">
-          <color rgb="FF002060"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color rgb="FF002060"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF002060"/>
-        </right>
-        <top style="hair">
-          <color rgb="FF002060"/>
-        </top>
-        <bottom style="hair">
-          <color rgb="FF002060"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color rgb="FF002060"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF002060"/>
-        </right>
-        <top style="hair">
-          <color rgb="FF002060"/>
-        </top>
-        <bottom style="hair">
-          <color rgb="FF002060"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="45">
     <dxf>
       <fill>
         <patternFill>
@@ -1983,49 +1898,49 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BCF95067-B771-3C4D-AD63-C29CB67B4C88}" name="Tabla1" displayName="Tabla1" ref="A4:AN54" totalsRowShown="0" dataDxfId="49" dataCellStyle="Millares">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BCF95067-B771-3C4D-AD63-C29CB67B4C88}" name="Tabla1" displayName="Tabla1" ref="A4:AN54" totalsRowShown="0" dataDxfId="44" dataCellStyle="Millares">
   <autoFilter ref="A4:AN54" xr:uid="{BCF95067-B771-3C4D-AD63-C29CB67B4C88}"/>
   <tableColumns count="40">
-    <tableColumn id="1" xr3:uid="{1B45D68F-9E92-9A48-B147-43382D17EADB}" name="Dir / Zona" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{8141432D-DFE6-034B-8474-F9783519965C}" name="Oficina" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{3026117E-099F-6549-A16F-3CA4F85DA282}" name="Mat" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{80621F5B-C573-8944-AF37-DC364F1BE0A9}" name="Suc" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{9D7D11D1-2D98-5646-92D8-F8703E85240A}" name="Promotor / Partner" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{870F3B42-A14B-1947-827D-9A6082152D25}" name="Asesor" dataDxfId="43"/>
-    <tableColumn id="7" xr3:uid="{CA38BEAA-FBC9-474E-8C66-960105DEBCF2}" name="Nombre del Asesor" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{8B8898BF-4E49-0543-9598-18FF2D3F6340}" name="Conexión" dataDxfId="41"/>
-    <tableColumn id="9" xr3:uid="{49ED1251-337D-EC49-A858-207AB60B673C}" name="Grupo" dataDxfId="40" dataCellStyle="Millares"/>
-    <tableColumn id="10" xr3:uid="{26692A66-EA2C-DD40-AAC8-07A5FE32BC7D}" name="Vida Individual" dataDxfId="39" dataCellStyle="Millares"/>
-    <tableColumn id="11" xr3:uid="{45DC445E-D43B-394B-91CD-B3001CC307CC}" name="Vida G&amp;C" dataDxfId="38" dataCellStyle="Millares"/>
-    <tableColumn id="12" xr3:uid="{953B1F2A-AB88-8A40-B82F-B5DBE8FAEA70}" name="Segudescuento" dataDxfId="37" dataCellStyle="Millares"/>
-    <tableColumn id="13" xr3:uid="{27E03CF4-3925-2045-BF66-C5BB1ECC7061}" name="Aportaciones Adicionales (AVEs)" dataDxfId="36" dataCellStyle="Millares"/>
-    <tableColumn id="14" xr3:uid="{7375183C-90AB-0B47-A516-65079E7802F1}" name="Cancelacion de Pólizas" dataDxfId="35" dataCellStyle="Millares"/>
-    <tableColumn id="15" xr3:uid="{B0F3DBFB-9B00-894E-8929-BF5CA63336C6}" name="Total de Productos Ilimitados" dataDxfId="34" dataCellStyle="Millares"/>
-    <tableColumn id="16" xr3:uid="{3C9D5C71-B64C-434C-8D65-968245DAE09C}" name="%Vida vs Meta" dataDxfId="33" dataCellStyle="Porcentaje"/>
-    <tableColumn id="17" xr3:uid="{088A86A3-8B28-DE4E-A384-CA0EA913DA34}" name="GMM Individual" dataDxfId="32" dataCellStyle="Millares"/>
-    <tableColumn id="18" xr3:uid="{A8791E9D-69D9-C844-AE4C-8AEEFA976B8B}" name="GMM G&amp;C" dataDxfId="31" dataCellStyle="Millares"/>
-    <tableColumn id="19" xr3:uid="{0FFCB5A1-F8D9-2344-9DC7-667454959C98}" name="Cancelacion de Pólizas2" dataDxfId="30" dataCellStyle="Millares"/>
-    <tableColumn id="20" xr3:uid="{FDCA43A0-92B9-954B-B283-ABAD7C194405}" name="Total Productos Limitados" dataDxfId="29" dataCellStyle="Millares"/>
-    <tableColumn id="21" xr3:uid="{7C93BB8B-9213-EA49-A648-EF5192999BF7}" name="Tope personales" dataDxfId="28" dataCellStyle="Millares"/>
-    <tableColumn id="22" xr3:uid="{70D3FAB6-79FB-994B-AB69-F0BBB15C6AFD}" name="Total Prima" dataDxfId="27" dataCellStyle="Millares"/>
-    <tableColumn id="23" xr3:uid="{0E0D17EB-06B5-AF45-9773-7D3921FC5B9C}" name="Vida Individual3" dataDxfId="26" dataCellStyle="Millares"/>
-    <tableColumn id="24" xr3:uid="{2A25EC7F-F387-9948-8D9A-38BFD2316AB4}" name="Vida G&amp;C4" dataDxfId="25" dataCellStyle="Millares"/>
-    <tableColumn id="25" xr3:uid="{F7E8005C-762C-7146-A541-3589C41B3DA2}" name="Segudescuento5" dataDxfId="24" dataCellStyle="Millares"/>
-    <tableColumn id="26" xr3:uid="{278BB65E-357A-1D4C-B1D0-5880BBD354CD}" name="Aportaciones Adicionales (AVEs)6" dataDxfId="23" dataCellStyle="Millares"/>
-    <tableColumn id="27" xr3:uid="{0490A388-0C84-C043-A7E8-E5DC8A03AF3F}" name="Cancelacion de Pólizas7" dataDxfId="22" dataCellStyle="Millares"/>
-    <tableColumn id="28" xr3:uid="{C06E1BE2-8968-A045-B8AB-E420B9B469A1}" name="Total de Productos Ilimitados8" dataDxfId="21" dataCellStyle="Millares"/>
-    <tableColumn id="29" xr3:uid="{BEBE08BA-F641-3141-BCA9-713FD1C7CEC2}" name="%Vida vs Meta9" dataDxfId="20" dataCellStyle="Porcentaje"/>
-    <tableColumn id="30" xr3:uid="{E7FB912B-27FD-1345-845F-E51E648031F5}" name="GMM Individual10" dataDxfId="19" dataCellStyle="Millares"/>
-    <tableColumn id="31" xr3:uid="{D5FF299C-A405-CE44-B4CD-CED400EFE81F}" name="GMM G&amp;C11" dataDxfId="18" dataCellStyle="Millares"/>
-    <tableColumn id="32" xr3:uid="{D7EFF89B-8E34-EA46-B72C-61EE3166E416}" name="Cancelacion de Pólizas12" dataDxfId="17" dataCellStyle="Millares"/>
-    <tableColumn id="33" xr3:uid="{81E1798B-3D20-E748-BDAB-7A2A6F5BF33B}" name="Total Productos Limitados13" dataDxfId="16" dataCellStyle="Millares"/>
-    <tableColumn id="34" xr3:uid="{7A820362-E31F-4D41-B400-9AD11AE00577}" name="Tope personales14" dataDxfId="15" dataCellStyle="Millares"/>
-    <tableColumn id="35" xr3:uid="{09E5F95B-08D0-B946-B14E-3F06BC9C57F0}" name="Total Comisión" dataDxfId="14" dataCellStyle="Millares"/>
-    <tableColumn id="36" xr3:uid="{523C81DC-6FA9-A24D-AF9B-9D74B552A8BA}" name="Columna15" dataDxfId="13" dataCellStyle="Millares"/>
-    <tableColumn id="37" xr3:uid="{ACF68D6F-CC4F-F94A-A3AE-C7407A1AC3DE}" name="Camino Prima" dataDxfId="12" dataCellStyle="Millares"/>
-    <tableColumn id="38" xr3:uid="{39FE9301-7AE9-0A42-B79D-CA4998AB76AE}" name="OBSERVACIÓN" dataDxfId="11" dataCellStyle="Millares"/>
-    <tableColumn id="39" xr3:uid="{99E25200-803C-E54D-88BD-27CB86CAED40}" name="Camino  Comisión" dataDxfId="10" dataCellStyle="Millares"/>
-    <tableColumn id="40" xr3:uid="{45B29C50-720D-8F4E-9803-310BA4AC814E}" name="NIVEL_x000a_" dataDxfId="9" dataCellStyle="Millares"/>
+    <tableColumn id="1" xr3:uid="{1B45D68F-9E92-9A48-B147-43382D17EADB}" name="Dir / Zona" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{8141432D-DFE6-034B-8474-F9783519965C}" name="Oficina" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{3026117E-099F-6549-A16F-3CA4F85DA282}" name="Mat" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{80621F5B-C573-8944-AF37-DC364F1BE0A9}" name="Suc" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{9D7D11D1-2D98-5646-92D8-F8703E85240A}" name="Promotor / Partner" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{870F3B42-A14B-1947-827D-9A6082152D25}" name="Asesor" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{CA38BEAA-FBC9-474E-8C66-960105DEBCF2}" name="Nombre del Asesor" dataDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{8B8898BF-4E49-0543-9598-18FF2D3F6340}" name="Conexión" dataDxfId="36"/>
+    <tableColumn id="9" xr3:uid="{49ED1251-337D-EC49-A858-207AB60B673C}" name="Grupo" dataDxfId="35" dataCellStyle="Millares"/>
+    <tableColumn id="10" xr3:uid="{26692A66-EA2C-DD40-AAC8-07A5FE32BC7D}" name="Vida Individual" dataDxfId="34" dataCellStyle="Millares"/>
+    <tableColumn id="11" xr3:uid="{45DC445E-D43B-394B-91CD-B3001CC307CC}" name="Vida G&amp;C" dataDxfId="33" dataCellStyle="Millares"/>
+    <tableColumn id="12" xr3:uid="{953B1F2A-AB88-8A40-B82F-B5DBE8FAEA70}" name="Segudescuento" dataDxfId="32" dataCellStyle="Millares"/>
+    <tableColumn id="13" xr3:uid="{27E03CF4-3925-2045-BF66-C5BB1ECC7061}" name="Aportaciones Adicionales (AVEs)" dataDxfId="31" dataCellStyle="Millares"/>
+    <tableColumn id="14" xr3:uid="{7375183C-90AB-0B47-A516-65079E7802F1}" name="Cancelacion de Pólizas" dataDxfId="30" dataCellStyle="Millares"/>
+    <tableColumn id="15" xr3:uid="{B0F3DBFB-9B00-894E-8929-BF5CA63336C6}" name="Total de Productos Ilimitados" dataDxfId="29" dataCellStyle="Millares"/>
+    <tableColumn id="16" xr3:uid="{3C9D5C71-B64C-434C-8D65-968245DAE09C}" name="%Vida vs Meta" dataDxfId="28" dataCellStyle="Porcentaje"/>
+    <tableColumn id="17" xr3:uid="{088A86A3-8B28-DE4E-A384-CA0EA913DA34}" name="GMM Individual" dataDxfId="27" dataCellStyle="Millares"/>
+    <tableColumn id="18" xr3:uid="{A8791E9D-69D9-C844-AE4C-8AEEFA976B8B}" name="GMM G&amp;C" dataDxfId="26" dataCellStyle="Millares"/>
+    <tableColumn id="19" xr3:uid="{0FFCB5A1-F8D9-2344-9DC7-667454959C98}" name="Cancelacion de Pólizas2" dataDxfId="25" dataCellStyle="Millares"/>
+    <tableColumn id="20" xr3:uid="{FDCA43A0-92B9-954B-B283-ABAD7C194405}" name="Total Productos Limitados" dataDxfId="24" dataCellStyle="Millares"/>
+    <tableColumn id="21" xr3:uid="{7C93BB8B-9213-EA49-A648-EF5192999BF7}" name="Tope personales" dataDxfId="23" dataCellStyle="Millares"/>
+    <tableColumn id="22" xr3:uid="{70D3FAB6-79FB-994B-AB69-F0BBB15C6AFD}" name="Total Prima" dataDxfId="22" dataCellStyle="Millares"/>
+    <tableColumn id="23" xr3:uid="{0E0D17EB-06B5-AF45-9773-7D3921FC5B9C}" name="Vida Individual3" dataDxfId="21" dataCellStyle="Millares"/>
+    <tableColumn id="24" xr3:uid="{2A25EC7F-F387-9948-8D9A-38BFD2316AB4}" name="Vida G&amp;C4" dataDxfId="20" dataCellStyle="Millares"/>
+    <tableColumn id="25" xr3:uid="{F7E8005C-762C-7146-A541-3589C41B3DA2}" name="Segudescuento5" dataDxfId="19" dataCellStyle="Millares"/>
+    <tableColumn id="26" xr3:uid="{278BB65E-357A-1D4C-B1D0-5880BBD354CD}" name="Aportaciones Adicionales (AVEs)6" dataDxfId="18" dataCellStyle="Millares"/>
+    <tableColumn id="27" xr3:uid="{0490A388-0C84-C043-A7E8-E5DC8A03AF3F}" name="Cancelacion de Pólizas7" dataDxfId="17" dataCellStyle="Millares"/>
+    <tableColumn id="28" xr3:uid="{C06E1BE2-8968-A045-B8AB-E420B9B469A1}" name="Total de Productos Ilimitados8" dataDxfId="16" dataCellStyle="Millares"/>
+    <tableColumn id="29" xr3:uid="{BEBE08BA-F641-3141-BCA9-713FD1C7CEC2}" name="%Vida vs Meta9" dataDxfId="15" dataCellStyle="Porcentaje"/>
+    <tableColumn id="30" xr3:uid="{E7FB912B-27FD-1345-845F-E51E648031F5}" name="GMM Individual10" dataDxfId="14" dataCellStyle="Millares"/>
+    <tableColumn id="31" xr3:uid="{D5FF299C-A405-CE44-B4CD-CED400EFE81F}" name="GMM G&amp;C11" dataDxfId="13" dataCellStyle="Millares"/>
+    <tableColumn id="32" xr3:uid="{D7EFF89B-8E34-EA46-B72C-61EE3166E416}" name="Cancelacion de Pólizas12" dataDxfId="12" dataCellStyle="Millares"/>
+    <tableColumn id="33" xr3:uid="{81E1798B-3D20-E748-BDAB-7A2A6F5BF33B}" name="Total Productos Limitados13" dataDxfId="11" dataCellStyle="Millares"/>
+    <tableColumn id="34" xr3:uid="{7A820362-E31F-4D41-B400-9AD11AE00577}" name="Tope personales14" dataDxfId="10" dataCellStyle="Millares"/>
+    <tableColumn id="35" xr3:uid="{09E5F95B-08D0-B946-B14E-3F06BC9C57F0}" name="Total Comisión" dataDxfId="9" dataCellStyle="Millares"/>
+    <tableColumn id="36" xr3:uid="{523C81DC-6FA9-A24D-AF9B-9D74B552A8BA}" name="Columna15" dataDxfId="8" dataCellStyle="Millares"/>
+    <tableColumn id="37" xr3:uid="{ACF68D6F-CC4F-F94A-A3AE-C7407A1AC3DE}" name="Camino Prima" dataDxfId="7" dataCellStyle="Millares"/>
+    <tableColumn id="38" xr3:uid="{39FE9301-7AE9-0A42-B79D-CA4998AB76AE}" name="OBSERVACIÓN" dataDxfId="6" dataCellStyle="Millares"/>
+    <tableColumn id="39" xr3:uid="{99E25200-803C-E54D-88BD-27CB86CAED40}" name="Camino  Comisión" dataDxfId="5" dataCellStyle="Millares"/>
+    <tableColumn id="40" xr3:uid="{45B29C50-720D-8F4E-9803-310BA4AC814E}" name="NIVEL_x000a_" dataDxfId="4" dataCellStyle="Millares"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7934,49 +7849,24 @@
       <c r="AN54" s="35"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A52:AI54 AM52:AN54 AK52:AK54">
-    <cfRule type="expression" dxfId="8" priority="10" stopIfTrue="1">
-      <formula>$B52&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK52:AN54">
-    <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
-      <formula>$B52&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL52:AL54">
-    <cfRule type="expression" dxfId="6" priority="8" stopIfTrue="1">
-      <formula>$B52&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AN52:AN54 V52:V54 AI52:AI54">
-    <cfRule type="expression" dxfId="5" priority="9" stopIfTrue="1">
-      <formula>$B52&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6:AI51 AK6:AK51 AM6:AN51">
-    <cfRule type="expression" dxfId="4" priority="5" stopIfTrue="1">
+  <conditionalFormatting sqref="A6:AI54 AM6:AN54 AK6:AK54">
+    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:V51 AI6:AI51 AN6:AN51">
-    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
+  <conditionalFormatting sqref="AK46:AN54">
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
+      <formula>$B46&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL6:AL54">
+    <cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AL6:AL51">
-    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
+  <conditionalFormatting sqref="AN6:AN54 V6:V54 AI6:AI54">
+    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK46:AN46">
-    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
-      <formula>$B46&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK47:AN51">
-    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>$B47&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>